<commit_message>
Updating questions to Hugo's last version and updating code to read questions from the 1st row in Excel
</commit_message>
<xml_diff>
--- a/questions_v3v2_hugo.xlsx
+++ b/questions_v3v2_hugo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10514"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jlbkm/document-tagging/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jlbkm\Coding\document-tagging\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7274F868-DE9F-5C4E-B771-D0F784AEA5B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5FBA6F2-A538-47F7-921B-EF1A06511644}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5340" yWindow="3380" windowWidth="27780" windowHeight="17780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="660" yWindow="1410" windowWidth="29520" windowHeight="15550" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Q_FOR_SCRIPT" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 1) Indicators used to assess the impact/outcome of CGIAR interventions,
 2) Units used to measure results, 
 3) The quantitative or qualitative results of the intervention. 
-Only capture these triplets if the numeric results are reported as statistically significant in the text. If multiple triplets are mentioned, output each as a list of three elements. For other significant or notable results (both quantitative or qualitative information that seems significant or relevant, although technically not statistically significant or not explicitly mentioned) capture them as a separate set of triples [Indicator, Units, Results].
+Only capture these triplets if the numeric results are reported as statistically significant in the text. If multiple triplets are mentioned, output each as a list of three elements. For other significant or notable results (both quantitative or qualitative information that seems significant or relevant, although technically not statistically significant or not explicitly mentioned) capture them as a separate set of triples [Indicator, Units, Results]. You should start your analysis by screening the sections "Abstract" or "Conclusion" (or similar sections) and based on the findings  you could extend the search to other sections from the study to complete your search.
 **Output Format:** 
 - Return a list of lists, with each nested list containing exactly three items in the order: [Indicator, Units, Results].
 - Separate each nested list with a comma. 
@@ -55,24 +55,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="&quot;Aptos Narrow&quot;"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -96,15 +83,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -326,20 +307,16 @@
     <tabColor rgb="FFF1C232"/>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.3984375" defaultRowHeight="15.75" customHeight="1"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="14.3984375" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="68" customWidth="1"/>
+    <col min="1" max="1" width="68" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A1" s="1"/>
-    </row>
-    <row r="2" spans="1:2" ht="409.5" customHeight="1">
-      <c r="A2" s="3" t="s">
+    <row r="1" spans="1:1" ht="409.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>